<commit_message>
Patch whatsapp-web.js for markedUnread error and force stable web version
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B101"/>
+  <dimension ref="A1:B103"/>
   <sheetData>
     <row r="1" xml:space="preserve">
       <c r="A1" t="str">
@@ -1729,9 +1729,31 @@
 </v>
       </c>
     </row>
+    <row r="102" xml:space="preserve">
+      <c r="A102" t="str">
+        <v>What is lumpy skin disease</v>
+      </c>
+      <c r="B102" t="str" xml:space="preserve">
+        <v xml:space="preserve">Based on our FAQ database:
+**Q:** What are the symptoms of fungal disease in fish?
+**A:** The skin looks like a white thread on the skin.
+_Note: AI assistance is currently unavailable. This is a direct FAQ match._</v>
+      </c>
+    </row>
+    <row r="103" xml:space="preserve">
+      <c r="A103" t="str">
+        <v>What are the symptoms of fungal disease in fish?</v>
+      </c>
+      <c r="B103" t="str" xml:space="preserve">
+        <v xml:space="preserve">Based on our FAQ database:
+**Q:** What are the symptoms of fungal disease in fish?
+**A:** The skin looks like a white thread on the skin.
+_Note: AI assistance is currently unavailable. This is a direct FAQ match._</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B101"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B103"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>